<commit_message>
added excel import and auth
</commit_message>
<xml_diff>
--- a/public/assets/syringe-filter.xlsx
+++ b/public/assets/syringe-filter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{35F8D584-918C-491D-AC0B-39205255496E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D473A3-E98C-43C2-9F42-98190B88596C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{316DEF0D-636A-47DB-8362-21A7012C13FB}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
   <si>
     <t>productName</t>
   </si>
@@ -129,6 +129,9 @@
   </si>
   <si>
     <t>OM268-020-GS</t>
+  </si>
+  <si>
+    <t>catalogueNumber Version</t>
   </si>
 </sst>
 </file>
@@ -495,28 +498,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{521DB8F3-95E8-4D16-8589-22BB2DB9755F}">
-  <dimension ref="A4:P6"/>
+  <dimension ref="A4:Q6"/>
   <sheetFormatPr defaultColWidth="56.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="39.28515625" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" customWidth="1"/>
-    <col min="7" max="7" width="37.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" customWidth="1"/>
-    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.140625" customWidth="1"/>
-    <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.140625" customWidth="1"/>
-    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="23.85546875" customWidth="1"/>
+    <col min="3" max="4" width="23.42578125" customWidth="1"/>
+    <col min="5" max="5" width="32.42578125" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="8" max="8" width="37.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" customWidth="1"/>
+    <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.140625" customWidth="1"/>
+    <col min="15" max="15" width="15" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -530,43 +533,46 @@
         <v>6</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="M4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="N4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="O4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="P4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="P4" s="3" t="s">
+      <c r="Q4" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -580,43 +586,46 @@
         <v>26</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="1">
+      <c r="J5" s="1">
         <v>100</v>
       </c>
-      <c r="J5" s="1">
+      <c r="K5" s="1">
         <v>84212900</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="M5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="M5" s="1">
+      <c r="N5" s="1">
         <v>25</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="P5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="P5" s="1" t="s">
+      <c r="Q5" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -627,42 +636,45 @@
         <v>5</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="1">
+      <c r="J6" s="1">
         <v>100</v>
       </c>
-      <c r="J6" s="1">
+      <c r="K6" s="1">
         <v>84212900</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="M6" s="1">
+      <c r="N6" s="1">
         <v>25</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="P6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="P6" s="1" t="s">
+      <c r="Q6" s="1" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>